<commit_message>
Replace full Application Profile clone with live FK model.
Configuration-related fields stay on the profile and apply to existing
Applications; per-Application fields keep defaults-only seeding from Excel E–H.

Co-authored-by: webapis <webapis@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/prototypes/Application-profile-wizard-draft.xlsx
+++ b/docs/prototypes/Application-profile-wizard-draft.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://calikholding-my.sharepoint.com/personal/serdar_asirow_gapinsaat_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webap\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="467" documentId="11_F25DC773A252ABDACC104812519E64445BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9D597FC-D846-4CFB-8A62-B9BE4AE46C73}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D083235B-15FD-4C8B-B9C4-1D22021A24D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="93">
   <si>
     <t>Application Related to :</t>
   </si>
@@ -303,6 +303,18 @@
   </si>
   <si>
     <t>APPLICATION TEPLATE RELATED CONFIGURATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editable Per Application. Persistent Per Application </t>
+  </si>
+  <si>
+    <t>Configuration Related</t>
+  </si>
+  <si>
+    <t>Only Per Application Related</t>
+  </si>
+  <si>
+    <t>Visibility on Application</t>
   </si>
 </sst>
 </file>
@@ -380,20 +392,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,330 +703,659 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:D106"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:H106"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.140625" customWidth="1"/>
-    <col min="2" max="2" width="49.5703125" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
+    <col min="2" max="2" width="49.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" customWidth="1"/>
+    <col min="4" max="4" width="27.54296875" style="12" customWidth="1"/>
+    <col min="5" max="5" width="22.7265625" customWidth="1"/>
+    <col min="6" max="6" width="31" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" customWidth="1"/>
+    <col min="8" max="8" width="15.08984375" customWidth="1"/>
+    <col min="9" max="9" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" s="10"/>
+      <c r="E5" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="10"/>
+      <c r="E6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="10"/>
+      <c r="E7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" s="10"/>
+      <c r="E8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" s="10"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" s="10"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="10"/>
+      <c r="E11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="10"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" s="10"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" s="10"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="10"/>
+      <c r="E15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="10"/>
+      <c r="E16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="10"/>
+      <c r="E17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="10"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="10"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D20" s="10"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D21" s="10"/>
+      <c r="E21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D22" s="10"/>
+      <c r="E22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" s="10"/>
+      <c r="E23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="10"/>
+      <c r="E24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" s="10"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="1"/>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="10"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D27" s="10"/>
+      <c r="E27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="10"/>
+      <c r="E28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D29" s="10"/>
+      <c r="E29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D30" s="10"/>
+      <c r="E30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="10"/>
+      <c r="E31" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4"/>
-      <c r="B33" s="9" t="s">
+      <c r="D32" s="10"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="3"/>
+      <c r="B33" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B34" s="10" t="s">
+      <c r="C33" s="4"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="10" t="s">
+      <c r="C34" s="3"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H34" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B36" s="10" t="s">
+      <c r="C35" s="3"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H35" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B37" s="10" t="s">
+      <c r="C36" s="3"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H36" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="C37" s="3"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H37" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="2"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C38" s="3"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H38" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="2"/>
       <c r="B41" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C41" s="1"/>
-      <c r="D41" s="1" t="s">
+      <c r="D41" s="11" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -1010,11 +1365,23 @@
       <c r="C42" t="s">
         <v>63</v>
       </c>
-      <c r="D42" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D42" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>62</v>
       </c>
@@ -1024,11 +1391,23 @@
       <c r="C43" t="s">
         <v>63</v>
       </c>
-      <c r="D43" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D43" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>62</v>
       </c>
@@ -1038,11 +1417,23 @@
       <c r="C44" t="s">
         <v>63</v>
       </c>
-      <c r="D44" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E44" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>62</v>
       </c>
@@ -1052,11 +1443,23 @@
       <c r="C45" t="s">
         <v>63</v>
       </c>
-      <c r="D45" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D45" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E45" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G45" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>62</v>
       </c>
@@ -1066,11 +1469,23 @@
       <c r="C46" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D46" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E46" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>62</v>
       </c>
@@ -1080,11 +1495,23 @@
       <c r="C47" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D47" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E47" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G47" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>62</v>
       </c>
@@ -1094,11 +1521,23 @@
       <c r="C48" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D48" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G48" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>62</v>
       </c>
@@ -1108,11 +1547,23 @@
       <c r="C49" t="s">
         <v>63</v>
       </c>
-      <c r="D49" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E49" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F49" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G49" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H49" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>62</v>
       </c>
@@ -1122,11 +1573,23 @@
       <c r="C50" t="s">
         <v>63</v>
       </c>
-      <c r="D50" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D50" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G50" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>62</v>
       </c>
@@ -1136,11 +1599,23 @@
       <c r="C51" t="s">
         <v>63</v>
       </c>
-      <c r="D51" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D51" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E51" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F51" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G51" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>62</v>
       </c>
@@ -1150,11 +1625,23 @@
       <c r="C52" t="s">
         <v>63</v>
       </c>
-      <c r="D52" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D52" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H52" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>62</v>
       </c>
@@ -1164,49 +1651,97 @@
       <c r="C53" t="s">
         <v>63</v>
       </c>
-      <c r="D53" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D53" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G53" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>62</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D54" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D54" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G54" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H54" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>62</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C55" t="s">
         <v>63</v>
       </c>
-      <c r="D55" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D55" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E55" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G55" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="2"/>
       <c r="B58" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C58" s="1"/>
-      <c r="D58" s="1" t="s">
+      <c r="D58" s="11" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E58" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F58" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G58" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H58" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>63</v>
       </c>
@@ -1214,11 +1749,23 @@
         <v>46</v>
       </c>
       <c r="C59" s="2"/>
-      <c r="D59" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D59" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E59" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G59" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>63</v>
       </c>
@@ -1226,115 +1773,223 @@
         <v>47</v>
       </c>
       <c r="C60" s="2"/>
-      <c r="D60" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="6" t="s">
+      <c r="D60" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G60" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H60" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A63" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+    </row>
+    <row r="65" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C65" s="7"/>
-      <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C65" s="1"/>
+      <c r="D65" s="10"/>
+      <c r="E65" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F65" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G65" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H65" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="2"/>
       <c r="B66" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C66" s="8"/>
-      <c r="D66" s="2"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C66" s="2"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F66" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G66" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="2"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D68" s="2"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C67" s="6"/>
+      <c r="D67" s="10"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D68" s="10"/>
+    </row>
+    <row r="69" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A69" s="2"/>
       <c r="B69" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C69" s="7" t="s">
+      <c r="C69" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D69" s="10"/>
+      <c r="E69" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F69" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G69" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H69" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C70" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="D70" s="2"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C70" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D70" s="10"/>
+      <c r="E70" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C71" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C71" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D71" s="10"/>
+      <c r="E71" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G71" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H71" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C72" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="D72" s="2"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C72" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D72" s="10"/>
+      <c r="E72" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F72" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G72" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H72" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C73" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="D73" s="2"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C73" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D73" s="10"/>
+      <c r="E73" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H73" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C74" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="D74" s="2"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C74" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D74" s="10"/>
+      <c r="E74" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H74" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A77" s="2"/>
       <c r="B77" s="1" t="s">
         <v>72</v>
@@ -1342,9 +1997,21 @@
       <c r="C77" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D77" s="2"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D77" s="10"/>
+      <c r="E77" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F77" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G77" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H77" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>62</v>
       </c>
@@ -1354,9 +2021,21 @@
       <c r="C78" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D78" s="2"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D78" s="10"/>
+      <c r="E78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G78" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H78" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>62</v>
       </c>
@@ -1366,9 +2045,21 @@
       <c r="C79" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D79" s="2"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D79" s="10"/>
+      <c r="E79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G79" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H79" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>62</v>
       </c>
@@ -1378,9 +2069,21 @@
       <c r="C80" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="D80" s="2"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D80" s="10"/>
+      <c r="E80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G80" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H80" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>62</v>
       </c>
@@ -1390,9 +2093,21 @@
       <c r="C81" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="D81" s="2"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D81" s="10"/>
+      <c r="E81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G81" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H81" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>62</v>
       </c>
@@ -1402,9 +2117,21 @@
       <c r="C82" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="D82" s="2"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D82" s="10"/>
+      <c r="E82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G82" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H82" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>62</v>
       </c>
@@ -1414,9 +2141,21 @@
       <c r="C83" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="D83" s="2"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D83" s="10"/>
+      <c r="E83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G83" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H83" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>62</v>
       </c>
@@ -1426,17 +2165,41 @@
       <c r="C84" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="D84" s="2"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D84" s="10"/>
+      <c r="E84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G84" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H84" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="2"/>
       <c r="B86" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C86" s="1"/>
-      <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D86" s="10"/>
+      <c r="E86" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F86" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G86" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H86" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>69</v>
       </c>
@@ -1444,9 +2207,21 @@
         <v>48</v>
       </c>
       <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D87" s="10"/>
+      <c r="E87" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F87" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G87" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H87" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>69</v>
       </c>
@@ -1454,17 +2229,29 @@
         <v>49</v>
       </c>
       <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="6" t="s">
+      <c r="D88" s="10"/>
+      <c r="E88" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F88" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G88" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H88" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A91" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B91" s="6"/>
-      <c r="C91" s="6"/>
-      <c r="D91" s="6"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B91" s="9"/>
+      <c r="C91" s="9"/>
+      <c r="D91" s="9"/>
+    </row>
+    <row r="93" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>65</v>
       </c>
@@ -1472,9 +2259,21 @@
         <v>41</v>
       </c>
       <c r="C93" s="1"/>
-      <c r="D93" s="2"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D93" s="10"/>
+      <c r="E93" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F93" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G93" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H93" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>66</v>
       </c>
@@ -1482,9 +2281,21 @@
         <v>42</v>
       </c>
       <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D94" s="10"/>
+      <c r="E94" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F94" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G94" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H94" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>67</v>
       </c>
@@ -1492,9 +2303,21 @@
         <v>43</v>
       </c>
       <c r="C95" s="2"/>
-      <c r="D95" s="2"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D95" s="10"/>
+      <c r="E95" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F95" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G95" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H95" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>68</v>
       </c>
@@ -1502,25 +2325,49 @@
         <v>44</v>
       </c>
       <c r="C96" s="2"/>
-      <c r="D96" s="2"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="6" t="s">
+      <c r="D96" s="10"/>
+      <c r="E96" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F96" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G96" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H96" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A99" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B99" s="9"/>
+      <c r="C99" s="9"/>
+      <c r="D99" s="9"/>
+    </row>
+    <row r="102" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A102" s="2"/>
       <c r="B102" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C102" s="2"/>
-      <c r="D102" s="2"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D102" s="10"/>
+      <c r="E102" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F102" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G102" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H102" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>62</v>
       </c>
@@ -1528,9 +2375,21 @@
         <v>53</v>
       </c>
       <c r="C103" s="2"/>
-      <c r="D103" s="2"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D103" s="10"/>
+      <c r="E103" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F103" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G103" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H103" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>62</v>
       </c>
@@ -1538,9 +2397,21 @@
         <v>54</v>
       </c>
       <c r="C104" s="2"/>
-      <c r="D104" s="2"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D104" s="10"/>
+      <c r="E104" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F104" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G104" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H104" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>62</v>
       </c>
@@ -1548,9 +2419,21 @@
         <v>55</v>
       </c>
       <c r="C105" s="2"/>
-      <c r="D105" s="2"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D105" s="10"/>
+      <c r="E105" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F105" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G105" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H105" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>62</v>
       </c>
@@ -1558,7 +2441,19 @@
         <v>56</v>
       </c>
       <c r="C106" s="2"/>
-      <c r="D106" s="2"/>
+      <c r="D106" s="10"/>
+      <c r="E106" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F106" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G106" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H106" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>